<commit_message>
Update - png flujo de trabajo
</commit_message>
<xml_diff>
--- a/docs/A2_llave_class_uso/Propuesta_clasificacion_llave_v2.xlsx
+++ b/docs/A2_llave_class_uso/Propuesta_clasificacion_llave_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesus\Work\CR\Github\PGBM_actividad_1_diagnostico\docs\A2_llave_class_uso\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{252060A5-3110-41A5-A3A2-2091EE38B928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78362C1E-05C4-4B66-AE38-B1043F1C5750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="homologacion_propuesta" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="138">
   <si>
     <t>Homologación propuesta: leyenda documental → leyenda propuesta</t>
   </si>
@@ -434,6 +434,12 @@
   </si>
   <si>
     <t>Humedales.</t>
+  </si>
+  <si>
+    <t>Árboles fuera de bosque y otras áreas naturales</t>
+  </si>
+  <si>
+    <t>Es una clase díficil de considerar como bosques y su predicción por tanto fue enviada a "Otras tierras"</t>
   </si>
 </sst>
 </file>
@@ -766,15 +772,92 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -790,84 +873,6 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -878,6 +883,317 @@
         <left style="thin">
           <color indexed="64"/>
         </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
         <right/>
         <top style="thin">
           <color indexed="64"/>
@@ -936,6 +1252,40 @@
       </border>
     </dxf>
     <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border>
         <bottom style="thin">
           <color indexed="64"/>
@@ -950,353 +1300,8 @@
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
         <top/>
         <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
         <vertical style="thin">
           <color indexed="64"/>
         </vertical>
@@ -1319,32 +1324,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1B5EE670-F716-40E1-AF68-5803BF26E340}" name="TablaHomologacion" displayName="TablaHomologacion" ref="A4:M43" headerRowDxfId="7" headerRowBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1B5EE670-F716-40E1-AF68-5803BF26E340}" name="TablaHomologacion" displayName="TablaHomologacion" ref="A4:M44" headerRowDxfId="14" headerRowBorderDxfId="13">
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{FA3617B9-DD08-466E-A7B5-0F891A09810E}" name="id_0_doc" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{DE595C6A-17F4-4F38-9196-CCE29F70D79D}" name="nivel_0_doc" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{FAB766C7-0F99-439F-9C8F-6D136FCFA2CE}" name="id_1_doc" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{5C5CA504-87E3-4A36-83B3-32B3A176D231}" name="nivel_1_doc" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{DFCD3B45-53EE-40D0-B8F7-2D3E9F279485}" name="id_2_doc" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{B1C603B8-832D-4144-AC3E-262F48E6CE7D}" name="nivel_2_doc" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{2FF22F72-4205-4EAF-967E-9FA694877803}" name="id_0_prop" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{42DAE2BF-6297-4DBD-BA30-364C060B4F4A}" name="nivel_0_prop" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{F318973E-93F5-4702-BA72-817D8083C146}" name="id_1_prop" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{CED329EF-DC4E-44D6-A65F-B5089E498F3E}" name="nivel_1_prop" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{2C5FAB4E-48C0-4291-A78B-8C687CA3DEE0}" name="tipo_criterio" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{3266DA6B-43D5-40CA-86C2-DA026EFED490}" name="criterio_homologación" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{2DCE3D2C-59E0-4A87-84E3-727E5E19CEDD}" name="observación" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{FA3617B9-DD08-466E-A7B5-0F891A09810E}" name="id_0_doc" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{DE595C6A-17F4-4F38-9196-CCE29F70D79D}" name="nivel_0_doc" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{FAB766C7-0F99-439F-9C8F-6D136FCFA2CE}" name="id_1_doc" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{5C5CA504-87E3-4A36-83B3-32B3A176D231}" name="nivel_1_doc" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{DFCD3B45-53EE-40D0-B8F7-2D3E9F279485}" name="id_2_doc" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{B1C603B8-832D-4144-AC3E-262F48E6CE7D}" name="nivel_2_doc" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{2FF22F72-4205-4EAF-967E-9FA694877803}" name="id_0_prop" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{42DAE2BF-6297-4DBD-BA30-364C060B4F4A}" name="nivel_0_prop" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{F318973E-93F5-4702-BA72-817D8083C146}" name="id_1_prop" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{CED329EF-DC4E-44D6-A65F-B5089E498F3E}" name="nivel_1_prop" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{2C5FAB4E-48C0-4291-A78B-8C687CA3DEE0}" name="tipo_criterio" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{3266DA6B-43D5-40CA-86C2-DA026EFED490}" name="criterio_homologación" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{2DCE3D2C-59E0-4A87-84E3-727E5E19CEDD}" name="observación" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8ED9CC01-582D-43B4-8020-43F8E0E96032}" name="TablaResumenDistribucion" displayName="TablaResumenDistribucion" ref="A11:C21" headerRowDxfId="6" totalsRowDxfId="5" headerRowBorderDxfId="3" tableBorderDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8ED9CC01-582D-43B4-8020-43F8E0E96032}" name="TablaResumenDistribucion" displayName="TablaResumenDistribucion" ref="A11:C21" headerRowDxfId="21" totalsRowDxfId="18" headerRowBorderDxfId="20" tableBorderDxfId="19">
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{DE029B88-F3FD-49B4-B828-92DBA3CC440B}" name="id_1_prop" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{FD2742B8-A722-42F8-A8EB-0A98A44E88BD}" name="nivel_1_prop" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{F4F7628C-0847-4E8F-BE3A-B78FECB95E4B}" name="n_clases_doc" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{DE029B88-F3FD-49B4-B828-92DBA3CC440B}" name="id_1_prop" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{FD2742B8-A722-42F8-A8EB-0A98A44E88BD}" name="nivel_1_prop" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{F4F7628C-0847-4E8F-BE3A-B78FECB95E4B}" name="n_clases_doc" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1613,7 +1618,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
@@ -1632,1647 +1637,1686 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="7"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
+      <c r="L2" s="38"/>
+      <c r="M2" s="38"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="9" t="s">
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="10" t="s">
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+      <c r="K3" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
+      <c r="L3" s="41"/>
+      <c r="M3" s="41"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="H4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="J4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="13" t="s">
+      <c r="K4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="13" t="s">
+      <c r="L4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="M4" s="13" t="s">
+      <c r="M4" s="7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>40</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <v>41</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>410</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <v>1</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>11</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="K5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="L5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="M5" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>40</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="1">
         <v>41</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>411</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="1">
         <v>1</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>11</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="K6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="L6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M6" s="2" t="s">
+      <c r="M6" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>40</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="1">
         <v>41</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>412</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="1">
         <v>1</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>11</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="K7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="L7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="M7" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>40</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="1">
         <v>41</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>413</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="1">
         <v>1</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>11</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="J8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="L8" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="M8" s="2"/>
+      <c r="M8" s="1"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>40</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="1">
         <v>44</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>441</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="1">
         <v>1</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>11</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="K9" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L9" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="M9" s="2"/>
+      <c r="M9" s="1"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>40</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="1">
         <v>44</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>444</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="1">
         <v>1</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>11</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="M10" s="2"/>
+      <c r="M10" s="1"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>40</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="1">
         <v>44</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>445</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="1">
         <v>1</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>11</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="J11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="K11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="L11" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="M11" s="2"/>
+      <c r="M11" s="1"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>40</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="1">
         <v>42</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>420</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="1">
         <v>1</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>12</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="J12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="K12" s="2" t="s">
+      <c r="K12" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L12" s="2" t="s">
+      <c r="L12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="M12" s="2"/>
+      <c r="M12" s="1"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>40</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="1">
         <v>42</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>421</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="1">
         <v>1</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>12</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="J13" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="K13" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L13" s="2" t="s">
+      <c r="L13" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="M13" s="2"/>
+      <c r="M13" s="1"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>40</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="1">
         <v>42</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>422</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="1">
         <v>1</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>12</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="J14" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="K14" s="2" t="s">
+      <c r="K14" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L14" s="2" t="s">
+      <c r="L14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="M14" s="2"/>
+      <c r="M14" s="1"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>40</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="1">
         <v>42</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>423</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="G15" s="2">
+      <c r="G15" s="1">
         <v>1</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>12</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="J15" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="K15" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L15" s="2" t="s">
+      <c r="L15" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="M15" s="2"/>
+      <c r="M15" s="1"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>40</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="1">
         <v>43</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>430</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G16" s="2">
+      <c r="G16" s="1">
         <v>1</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>13</v>
       </c>
-      <c r="J16" s="2" t="s">
+      <c r="J16" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="K16" s="2" t="s">
+      <c r="K16" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L16" s="2" t="s">
+      <c r="L16" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="M16" s="2"/>
+      <c r="M16" s="1"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>40</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17" s="1">
         <v>43</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>431</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G17" s="2">
+      <c r="G17" s="1">
         <v>1</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="H17" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>13</v>
       </c>
-      <c r="J17" s="2" t="s">
+      <c r="J17" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="K17" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L17" s="2" t="s">
+      <c r="L17" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="M17" s="2"/>
+      <c r="M17" s="1"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>40</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="1">
         <v>43</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>432</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G18" s="2">
+      <c r="G18" s="1">
         <v>1</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="H18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="2">
+      <c r="I18" s="1">
         <v>13</v>
       </c>
-      <c r="J18" s="2" t="s">
+      <c r="J18" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="K18" s="2" t="s">
+      <c r="K18" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L18" s="2" t="s">
+      <c r="L18" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="M18" s="2"/>
+      <c r="M18" s="1"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>40</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="1">
         <v>41</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>414</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="G19" s="2">
+      <c r="G19" s="1">
         <v>1</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H19" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I19" s="2">
+      <c r="I19" s="1">
         <v>14</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="J19" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="K19" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L19" s="2" t="s">
+      <c r="L19" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="M19" s="2"/>
+      <c r="M19" s="1"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>40</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="1">
         <v>44</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>442</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G20" s="2">
+      <c r="G20" s="1">
         <v>1</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="H20" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I20" s="2">
+      <c r="I20" s="1">
         <v>15</v>
       </c>
-      <c r="J20" s="2" t="s">
+      <c r="J20" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="K20" s="2" t="s">
+      <c r="K20" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L20" s="2" t="s">
+      <c r="L20" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="M20" s="2"/>
+      <c r="M20" s="1"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A21" s="3">
+      <c r="A21" s="2">
         <v>30</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21" s="2">
         <v>31</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E21" s="3">
+      <c r="E21" s="2">
         <v>311</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="F21" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G21" s="3">
+      <c r="G21" s="2">
         <v>2</v>
       </c>
-      <c r="H21" s="3" t="s">
+      <c r="H21" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I21" s="3">
+      <c r="I21" s="2">
         <v>21</v>
       </c>
-      <c r="J21" s="3" t="s">
+      <c r="J21" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="K21" s="3" t="s">
+      <c r="K21" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L21" s="3" t="s">
+      <c r="L21" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="M21" s="3"/>
+      <c r="M21" s="2"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" s="3">
+      <c r="A22" s="2">
         <v>30</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C22" s="2">
         <v>32</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E22" s="3">
+      <c r="E22" s="2">
         <v>321</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G22" s="3">
+      <c r="G22" s="2">
         <v>2</v>
       </c>
-      <c r="H22" s="3" t="s">
+      <c r="H22" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I22" s="3">
+      <c r="I22" s="2">
         <v>21</v>
       </c>
-      <c r="J22" s="3" t="s">
+      <c r="J22" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="K22" s="3" t="s">
+      <c r="K22" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L22" s="3" t="s">
+      <c r="L22" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="M22" s="3"/>
+      <c r="M22" s="2"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A23" s="3">
+      <c r="A23" s="2">
         <v>30</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C23" s="3">
+      <c r="C23" s="2">
         <v>32</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E23" s="3">
+      <c r="E23" s="2">
         <v>322</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G23" s="3">
+      <c r="G23" s="2">
         <v>2</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="H23" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I23" s="3">
+      <c r="I23" s="2">
         <v>21</v>
       </c>
-      <c r="J23" s="3" t="s">
+      <c r="J23" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="K23" s="3" t="s">
+      <c r="K23" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L23" s="3" t="s">
+      <c r="L23" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="M23" s="3"/>
+      <c r="M23" s="2"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A24" s="3">
+      <c r="A24" s="2">
         <v>30</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C24" s="3">
+      <c r="C24" s="2">
         <v>32</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E24" s="2">
         <v>323</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F24" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G24" s="3">
+      <c r="G24" s="2">
         <v>2</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="H24" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I24" s="3">
+      <c r="I24" s="2">
         <v>21</v>
       </c>
-      <c r="J24" s="3" t="s">
+      <c r="J24" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="K24" s="3" t="s">
+      <c r="K24" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L24" s="3" t="s">
+      <c r="L24" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="M24" s="3"/>
+      <c r="M24" s="2"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A25" s="3">
+      <c r="A25" s="2">
         <v>30</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="3">
+      <c r="C25" s="2">
         <v>32</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E25" s="3">
+      <c r="E25" s="2">
         <v>324</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="F25" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G25" s="3">
+      <c r="G25" s="2">
         <v>2</v>
       </c>
-      <c r="H25" s="3" t="s">
+      <c r="H25" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I25" s="3">
+      <c r="I25" s="2">
         <v>21</v>
       </c>
-      <c r="J25" s="3" t="s">
+      <c r="J25" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="K25" s="3" t="s">
+      <c r="K25" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L25" s="3" t="s">
+      <c r="L25" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="M25" s="3"/>
+      <c r="M25" s="2"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" s="3">
+      <c r="A26" s="2">
         <v>30</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="3">
+      <c r="C26" s="2">
         <v>32</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E26" s="2">
         <v>325</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="F26" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="G26" s="3">
+      <c r="G26" s="2">
         <v>2</v>
       </c>
-      <c r="H26" s="3" t="s">
+      <c r="H26" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I26" s="3">
+      <c r="I26" s="2">
         <v>21</v>
       </c>
-      <c r="J26" s="3" t="s">
+      <c r="J26" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="K26" s="3" t="s">
+      <c r="K26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L26" s="3" t="s">
+      <c r="L26" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="M26" s="3" t="s">
+      <c r="M26" s="2" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A27" s="3">
+      <c r="A27" s="2">
         <v>30</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C27" s="3">
+      <c r="C27" s="2">
         <v>31</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E27" s="3">
+      <c r="E27" s="2">
         <v>312</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="F27" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="G27" s="3">
+      <c r="G27" s="2">
         <v>2</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="H27" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I27" s="3">
+      <c r="I27" s="2">
         <v>22</v>
       </c>
-      <c r="J27" s="3" t="s">
+      <c r="J27" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="K27" s="3" t="s">
+      <c r="K27" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L27" s="3" t="s">
+      <c r="L27" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="M27" s="3"/>
+      <c r="M27" s="2"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A28" s="3">
+      <c r="A28" s="2">
         <v>30</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="3">
+      <c r="C28" s="2">
         <v>31</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E28" s="3">
+      <c r="E28" s="2">
         <v>313</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="F28" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="G28" s="3">
+      <c r="G28" s="2">
         <v>2</v>
       </c>
-      <c r="H28" s="3" t="s">
+      <c r="H28" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I28" s="3">
+      <c r="I28" s="2">
         <v>22</v>
       </c>
-      <c r="J28" s="3" t="s">
+      <c r="J28" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="K28" s="3" t="s">
+      <c r="K28" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L28" s="3" t="s">
+      <c r="L28" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="M28" s="3"/>
+      <c r="M28" s="2"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A29" s="3">
+      <c r="A29" s="2">
         <v>30</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="3">
+      <c r="C29" s="2">
         <v>31</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E29" s="3">
+      <c r="E29" s="2">
         <v>314</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="F29" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="G29" s="3">
+      <c r="G29" s="2">
         <v>2</v>
       </c>
-      <c r="H29" s="3" t="s">
+      <c r="H29" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I29" s="3">
+      <c r="I29" s="2">
         <v>22</v>
       </c>
-      <c r="J29" s="3" t="s">
+      <c r="J29" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="K29" s="3" t="s">
+      <c r="K29" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L29" s="3" t="s">
+      <c r="L29" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="M29" s="3"/>
+      <c r="M29" s="2"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A30" s="3">
+      <c r="A30" s="2">
         <v>30</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="3">
+      <c r="C30" s="2">
         <v>31</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E30" s="3">
+      <c r="E30" s="2">
         <v>315</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="F30" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="G30" s="3">
+      <c r="G30" s="2">
         <v>2</v>
       </c>
-      <c r="H30" s="3" t="s">
+      <c r="H30" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I30" s="3">
+      <c r="I30" s="2">
         <v>22</v>
       </c>
-      <c r="J30" s="3" t="s">
+      <c r="J30" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="K30" s="3" t="s">
+      <c r="K30" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L30" s="3" t="s">
+      <c r="L30" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="M30" s="3"/>
+      <c r="M30" s="2"/>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A31" s="3">
+      <c r="A31" s="2">
         <v>30</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C31" s="3">
+      <c r="C31" s="2">
         <v>33</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E31" s="3">
+      <c r="E31" s="2">
         <v>331</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="F31" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="G31" s="3">
+      <c r="G31" s="2">
         <v>2</v>
       </c>
-      <c r="H31" s="3" t="s">
+      <c r="H31" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I31" s="3">
+      <c r="I31" s="2">
         <v>22</v>
       </c>
-      <c r="J31" s="3" t="s">
+      <c r="J31" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="K31" s="3" t="s">
+      <c r="K31" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L31" s="3" t="s">
+      <c r="L31" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="M31" s="3"/>
+      <c r="M31" s="2"/>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A32" s="3">
+      <c r="A32" s="2">
         <v>30</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C32" s="2">
         <v>33</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E32" s="3">
+      <c r="E32" s="2">
         <v>332</v>
       </c>
-      <c r="F32" s="3" t="s">
+      <c r="F32" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G32" s="3">
+      <c r="G32" s="2">
         <v>2</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="H32" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I32" s="3">
+      <c r="I32" s="2">
         <v>22</v>
       </c>
-      <c r="J32" s="3" t="s">
+      <c r="J32" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="K32" s="3" t="s">
+      <c r="K32" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L32" s="3" t="s">
+      <c r="L32" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="M32" s="3" t="s">
+      <c r="M32" s="2" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A33" s="3">
+      <c r="A33" s="2">
         <v>30</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="3">
+      <c r="C33" s="2">
         <v>33</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E33" s="3">
+      <c r="E33" s="2">
         <v>333</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="F33" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="G33" s="3">
+      <c r="G33" s="2">
         <v>2</v>
       </c>
-      <c r="H33" s="3" t="s">
+      <c r="H33" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I33" s="3">
+      <c r="I33" s="2">
         <v>22</v>
       </c>
-      <c r="J33" s="3" t="s">
+      <c r="J33" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="K33" s="3" t="s">
+      <c r="K33" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L33" s="3" t="s">
+      <c r="L33" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="M33" s="3" t="s">
+      <c r="M33" s="2" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A34" s="3">
+      <c r="A34" s="2">
         <v>10</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C34" s="3">
+      <c r="C34" s="2">
         <v>11</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E34" s="3">
+      <c r="E34" s="2">
         <v>110</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="F34" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="G34" s="3">
+      <c r="G34" s="2">
         <v>2</v>
       </c>
-      <c r="H34" s="3" t="s">
+      <c r="H34" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I34" s="3">
+      <c r="I34" s="2">
         <v>23</v>
       </c>
-      <c r="J34" s="3" t="s">
+      <c r="J34" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="K34" s="3" t="s">
+      <c r="K34" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L34" s="3" t="s">
+      <c r="L34" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="M34" s="3" t="s">
+      <c r="M34" s="2" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A35" s="3">
+      <c r="A35" s="2">
         <v>10</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C35" s="3">
+      <c r="C35" s="2">
         <v>11</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E35" s="3">
+      <c r="E35" s="2">
         <v>111</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="F35" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="G35" s="3">
+      <c r="G35" s="2">
         <v>2</v>
       </c>
-      <c r="H35" s="3" t="s">
+      <c r="H35" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I35" s="3">
+      <c r="I35" s="2">
         <v>23</v>
       </c>
-      <c r="J35" s="3" t="s">
+      <c r="J35" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="K35" s="3" t="s">
+      <c r="K35" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L35" s="3" t="s">
+      <c r="L35" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="M35" s="3" t="s">
+      <c r="M35" s="2" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A36" s="3">
+      <c r="A36" s="2">
         <v>10</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C36" s="3">
+      <c r="C36" s="2">
         <v>11</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E36" s="3">
+      <c r="E36" s="2">
         <v>112</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="F36" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="G36" s="3">
+      <c r="G36" s="2">
         <v>2</v>
       </c>
-      <c r="H36" s="3" t="s">
+      <c r="H36" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I36" s="3">
+      <c r="I36" s="2">
         <v>23</v>
       </c>
-      <c r="J36" s="3" t="s">
+      <c r="J36" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="K36" s="3" t="s">
+      <c r="K36" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L36" s="3" t="s">
+      <c r="L36" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="M36" s="3" t="s">
+      <c r="M36" s="2" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A37" s="3">
+      <c r="A37" s="2">
         <v>10</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C37" s="3">
+      <c r="C37" s="2">
         <v>12</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E37" s="3">
+      <c r="E37" s="2">
         <v>121</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="F37" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="G37" s="3">
+      <c r="G37" s="2">
         <v>2</v>
       </c>
-      <c r="H37" s="3" t="s">
+      <c r="H37" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I37" s="3">
+      <c r="I37" s="2">
         <v>23</v>
       </c>
-      <c r="J37" s="3" t="s">
+      <c r="J37" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="K37" s="3" t="s">
+      <c r="K37" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L37" s="3" t="s">
+      <c r="L37" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="M37" s="3" t="s">
+      <c r="M37" s="2" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A38" s="3">
+      <c r="A38" s="2">
         <v>20</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C38" s="3">
+      <c r="C38" s="2">
         <v>21</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E38" s="3">
+      <c r="E38" s="2">
         <v>210</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="F38" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="G38" s="3">
+      <c r="G38" s="2">
         <v>2</v>
       </c>
-      <c r="H38" s="3" t="s">
+      <c r="H38" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I38" s="3">
+      <c r="I38" s="2">
         <v>24</v>
       </c>
-      <c r="J38" s="3" t="s">
+      <c r="J38" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="K38" s="3" t="s">
+      <c r="K38" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L38" s="3" t="s">
+      <c r="L38" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="M38" s="3"/>
+      <c r="M38" s="2"/>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A39" s="3">
+      <c r="A39" s="2">
         <v>20</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C39" s="3">
+      <c r="C39" s="2">
         <v>21</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E39" s="3">
+      <c r="E39" s="2">
         <v>211</v>
       </c>
-      <c r="F39" s="3" t="s">
+      <c r="F39" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="G39" s="3">
+      <c r="G39" s="2">
         <v>2</v>
       </c>
-      <c r="H39" s="3" t="s">
+      <c r="H39" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I39" s="3">
+      <c r="I39" s="2">
         <v>24</v>
       </c>
-      <c r="J39" s="3" t="s">
+      <c r="J39" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="K39" s="3" t="s">
+      <c r="K39" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L39" s="3" t="s">
+      <c r="L39" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="M39" s="3"/>
+      <c r="M39" s="2"/>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A40" s="3">
+      <c r="A40" s="2">
         <v>20</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="B40" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C40" s="3">
+      <c r="C40" s="2">
         <v>21</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E40" s="3">
+      <c r="E40" s="2">
         <v>212</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="F40" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="G40" s="3">
+      <c r="G40" s="2">
         <v>2</v>
       </c>
-      <c r="H40" s="3" t="s">
+      <c r="H40" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I40" s="3">
+      <c r="I40" s="2">
         <v>24</v>
       </c>
-      <c r="J40" s="3" t="s">
+      <c r="J40" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="K40" s="3" t="s">
+      <c r="K40" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L40" s="3" t="s">
+      <c r="L40" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="M40" s="3"/>
+      <c r="M40" s="2"/>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A41" s="3">
+      <c r="A41" s="2">
         <v>10</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B41" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C41" s="3">
+      <c r="C41" s="2">
         <v>12</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E41" s="3">
+      <c r="E41" s="2">
         <v>122</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="F41" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="G41" s="3">
+      <c r="G41" s="2">
         <v>2</v>
       </c>
-      <c r="H41" s="3" t="s">
+      <c r="H41" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I41" s="3">
+      <c r="I41" s="2">
         <v>25</v>
       </c>
-      <c r="J41" s="3" t="s">
+      <c r="J41" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="K41" s="3" t="s">
+      <c r="K41" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L41" s="3" t="s">
+      <c r="L41" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="M41" s="3" t="s">
+      <c r="M41" s="2" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A42" s="3">
+      <c r="A42" s="2">
         <v>20</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B42" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C42" s="3">
+      <c r="C42" s="2">
         <v>22</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E42" s="3">
+      <c r="E42" s="2">
         <v>220</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="F42" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G42" s="3">
+      <c r="G42" s="2">
         <v>2</v>
       </c>
-      <c r="H42" s="3" t="s">
+      <c r="H42" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I42" s="3">
+      <c r="I42" s="2">
         <v>25</v>
       </c>
-      <c r="J42" s="3" t="s">
+      <c r="J42" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="K42" s="39" t="s">
+      <c r="K42" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="L42" s="3" t="s">
+      <c r="L42" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="M42" s="39" t="s">
+      <c r="M42" s="32" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A43" s="3">
+      <c r="A43" s="2">
         <v>90</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C43" s="3">
+      <c r="C43" s="2">
         <v>91</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="E43" s="3">
+      <c r="E43" s="2">
         <v>910</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="F43" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="G43" s="3">
+      <c r="G43" s="2">
         <v>2</v>
       </c>
-      <c r="H43" s="3" t="s">
+      <c r="H43" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I43" s="3">
+      <c r="I43" s="2">
         <v>25</v>
       </c>
-      <c r="J43" s="3" t="s">
+      <c r="J43" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="K43" s="3" t="s">
+      <c r="K43" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L43" s="3" t="s">
+      <c r="L43" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="M43" s="3" t="s">
+      <c r="M43" s="2" t="s">
         <v>121</v>
       </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A44" s="2">
+        <v>40</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C44" s="2">
+        <v>44</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E44" s="2">
+        <v>443</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G44" s="2">
+        <v>2</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="I44" s="2">
+        <v>25</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="M44" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3304,41 +3348,41 @@
     <col min="8" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="K1" s="15"/>
-    </row>
-    <row r="2" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="K1" s="9"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="31" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="K2" s="19"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="K2" s="12"/>
     </row>
     <row r="4" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="F4" s="21" t="s">
         <v>127</v>
       </c>
     </row>
@@ -3347,12 +3391,12 @@
         <v>128</v>
       </c>
       <c r="B5">
-        <v>39</v>
-      </c>
-      <c r="E5" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="30">
+      <c r="F5" s="23">
         <v>27</v>
       </c>
     </row>
@@ -3363,11 +3407,11 @@
       <c r="B6">
         <v>16</v>
       </c>
-      <c r="E6" s="31" t="s">
+      <c r="E6" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="32">
-        <v>10</v>
+      <c r="F6" s="25">
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -3375,12 +3419,12 @@
         <v>130</v>
       </c>
       <c r="B7">
-        <v>23</v>
-      </c>
-      <c r="E7" s="33" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="34">
+      <c r="F7" s="27">
         <v>2</v>
       </c>
     </row>
@@ -3393,142 +3437,142 @@
       </c>
     </row>
     <row r="11" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="C11" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="E11" s="35" t="s">
+      <c r="E11" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="36" t="s">
+      <c r="F11" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="G11" s="37" t="s">
+      <c r="G11" s="30" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="23">
+      <c r="A12" s="16">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="24">
+      <c r="C12" s="17">
         <v>7</v>
       </c>
-      <c r="E12" s="40">
+      <c r="E12" s="33">
         <v>220</v>
       </c>
-      <c r="F12" s="41" t="s">
+      <c r="F12" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="G12" s="42" t="s">
+      <c r="G12" s="35" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="23">
+      <c r="A13" s="16">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="24">
+      <c r="C13" s="17">
         <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="23">
+      <c r="A14" s="16">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C14" s="24">
+      <c r="C14" s="17">
         <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="23">
+      <c r="A15" s="16">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="24">
+      <c r="C15" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="23">
+      <c r="A16" s="16">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="24">
+      <c r="C16" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="23">
+      <c r="A17" s="16">
         <v>21</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="24">
+      <c r="C17" s="17">
         <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="23">
+      <c r="A18" s="16">
         <v>22</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="24">
+      <c r="C18" s="17">
         <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="23">
+      <c r="A19" s="16">
         <v>23</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="17">
         <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="23">
+      <c r="A20" s="16">
         <v>24</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C20" s="24">
+      <c r="C20" s="17">
         <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="25">
+      <c r="A21" s="18">
         <v>25</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C21" s="26">
-        <v>3</v>
+      <c r="C21" s="19">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>